<commit_message>
Update rod selection demo pages
</commit_message>
<xml_diff>
--- a/pages/page11/rodfather/Rod-Father.xlsx
+++ b/pages/page11/rodfather/Rod-Father.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1480" yWindow="1640" windowWidth="23700" windowHeight="13840" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offcuts" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Offcuts" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData>
     <row r="1">
@@ -685,7 +685,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Available</t>
+          <t>Reserved</t>
         </is>
       </c>
     </row>
@@ -735,7 +735,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Available</t>
+          <t>Reserved</t>
         </is>
       </c>
     </row>
@@ -834,6 +834,56 @@
         <v>25</v>
       </c>
       <c r="E15" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>AUTO0015</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Cobalt Chrome</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Cylindrical</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>150</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>AUTO0016</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Titanium</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Hex</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>140</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>Available</t>
         </is>

</xml_diff>